<commit_message>
E3.1: harden Q2 trace and multiobjective validation
</commit_message>
<xml_diff>
--- a/results/q2/Q2_submission.xlsx
+++ b/results/q2/Q2_submission.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,17 +508,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>S007&gt;S006</t>
+          <t>S001&gt;S012</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2121.702052162075</v>
+        <v>2430.151333022899</v>
       </c>
       <c r="I2" t="n">
-        <v>2.188968719659792</v>
+        <v>3.091608697291146</v>
       </c>
       <c r="J2" t="n">
-        <v>1.411031280340208</v>
+        <v>0.508391302708854</v>
       </c>
       <c r="K2" t="n">
         <v>3</v>
@@ -556,17 +556,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>S001&gt;S012</t>
+          <t>S014&gt;S011</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2430.151333022899</v>
+        <v>2652.617556574498</v>
       </c>
       <c r="I3" t="n">
-        <v>3.091608697291146</v>
+        <v>3.189918429941903</v>
       </c>
       <c r="J3" t="n">
-        <v>0.508391302708854</v>
+        <v>0.4100815700580971</v>
       </c>
       <c r="K3" t="n">
         <v>3</v>
@@ -611,16 +611,16 @@
         <v>1560.170391878965</v>
       </c>
       <c r="I4" t="n">
-        <v>2.638536993772959</v>
+        <v>2.780626354602164</v>
       </c>
       <c r="J4" t="n">
-        <v>3.761463006227042</v>
+        <v>3.619373645397836</v>
       </c>
       <c r="K4" t="n">
         <v>7</v>
       </c>
       <c r="L4" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5">
@@ -652,17 +652,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>S014</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1869.752194619016</v>
+        <v>1816.693933921912</v>
       </c>
       <c r="I5" t="n">
-        <v>2.140303004761489</v>
+        <v>2.713392714678266</v>
       </c>
       <c r="J5" t="n">
-        <v>1.059696995238511</v>
+        <v>0.4866072853217345</v>
       </c>
       <c r="K5" t="n">
         <v>3</v>
@@ -679,44 +679,44 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>U06</t>
+          <t>U08</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>BAT-B-02</t>
+          <t>BAT-C-02</t>
         </is>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>390</v>
+        <v>480</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1816.693933921912</v>
+        <v>1494.170391878965</v>
       </c>
       <c r="I6" t="n">
-        <v>2.713392714678266</v>
+        <v>2.812680161939696</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4866072853217345</v>
+        <v>3.587319838060305</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L6" t="n">
-        <v>25</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7">
@@ -727,44 +727,44 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>U08</t>
+          <t>U03</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BAT-C-02</t>
+          <t>BAT-A-03</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>480</v>
+        <v>360</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1494.170391878965</v>
+        <v>1712.55936238718</v>
       </c>
       <c r="I7" t="n">
-        <v>2.995742764547403</v>
+        <v>1.899286069408222</v>
       </c>
       <c r="J7" t="n">
-        <v>3.404257235452597</v>
+        <v>1.700713930591778</v>
       </c>
       <c r="K7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>78</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -775,44 +775,44 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>U08</t>
+          <t>U04</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>BAT-C-03</t>
+          <t>BAT-A-04</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1494.170391878965</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>1944.170391878965</v>
+        <v>360</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S010</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>2989.729917819312</v>
+        <v>1654.859398321596</v>
       </c>
       <c r="I8" t="n">
-        <v>2.539471952043197</v>
+        <v>1.954809785440372</v>
       </c>
       <c r="J8" t="n">
-        <v>3.860528047956803</v>
+        <v>1.645190214559628</v>
       </c>
       <c r="K8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L8" t="n">
-        <v>56</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -823,7 +823,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>U03</t>
+          <t>U04</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -833,28 +833,28 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>BAT-A-03</t>
+          <t>BAT-A-05</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1654.859398321596</v>
       </c>
       <c r="F9" t="n">
-        <v>360</v>
+        <v>2014.859398321596</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>S010</t>
+          <t>S013</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1654.859398321596</v>
+        <v>3264.325987701448</v>
       </c>
       <c r="I9" t="n">
-        <v>1.954809785440372</v>
+        <v>1.956841224427769</v>
       </c>
       <c r="J9" t="n">
-        <v>1.645190214559628</v>
+        <v>1.643158775572231</v>
       </c>
       <c r="K9" t="n">
         <v>2</v>
@@ -871,17 +871,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>U04</t>
+          <t>U06</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>BAT-A-04</t>
+          <t>BAT-B-02</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -892,17 +892,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>S013</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1609.466589379853</v>
+        <v>1207.276912821857</v>
       </c>
       <c r="I10" t="n">
-        <v>1.956841224427769</v>
+        <v>1.098763738436815</v>
       </c>
       <c r="J10" t="n">
-        <v>1.643158775572231</v>
+        <v>2.101236261563185</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -919,44 +919,44 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U03</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>BAT-C-04</t>
+          <t>BAT-A-06</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1560.170391878965</v>
+        <v>1712.55936238718</v>
       </c>
       <c r="F11" t="n">
-        <v>2010.170391878965</v>
+        <v>2072.55936238718</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>3759.882476471139</v>
+        <v>3959.995061810809</v>
       </c>
       <c r="I11" t="n">
-        <v>5.836023632389955</v>
+        <v>2.97580685779325</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5639763676100458</v>
+        <v>0.6241931422067499</v>
       </c>
       <c r="K11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L11" t="n">
-        <v>45</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12">
@@ -981,24 +981,24 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1816.693933921912</v>
+        <v>1207.276912821857</v>
       </c>
       <c r="F12" t="n">
-        <v>2176.693933921912</v>
+        <v>1567.276912821857</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3822.018709443888</v>
+        <v>3128.924923995099</v>
       </c>
       <c r="I12" t="n">
-        <v>2.491188971973507</v>
+        <v>2.576489867036754</v>
       </c>
       <c r="J12" t="n">
-        <v>0.708811028026493</v>
+        <v>0.6235101329632462</v>
       </c>
       <c r="K12" t="n">
         <v>2</v>
@@ -1029,24 +1029,24 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1869.752194619016</v>
+        <v>1816.693933921912</v>
       </c>
       <c r="F13" t="n">
-        <v>2229.752194619016</v>
+        <v>2176.693933921912</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>3791.400205792258</v>
+        <v>3718.536241088956</v>
       </c>
       <c r="I13" t="n">
-        <v>2.576489867036754</v>
+        <v>2.667681609599494</v>
       </c>
       <c r="J13" t="n">
-        <v>0.6235101329632462</v>
+        <v>0.5323183904005058</v>
       </c>
       <c r="K13" t="n">
         <v>2</v>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>U05</t>
+          <t>U06</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1073,14 +1073,14 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>BAT-B-01</t>
+          <t>BAT-B-02</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>3791.400205792258</v>
+        <v>3128.924923995099</v>
       </c>
       <c r="F14" t="n">
-        <v>4181.400205792258</v>
+        <v>3518.924923995099</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1088,7 +1088,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>5618.325516700729</v>
+        <v>4955.85023490357</v>
       </c>
       <c r="I14" t="n">
         <v>2.306879693794434</v>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>U04</t>
+          <t>U01</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1121,28 +1121,28 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BAT-A-05</t>
+          <t>BAT-A-03</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1609.466589379853</v>
+        <v>2430.151333022899</v>
       </c>
       <c r="F15" t="n">
-        <v>1969.466589379853</v>
+        <v>2790.151333022899</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S009</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>3301.662840997978</v>
+        <v>4118.765207736287</v>
       </c>
       <c r="I15" t="n">
-        <v>2.12130507403894</v>
+        <v>2.254800043434852</v>
       </c>
       <c r="J15" t="n">
-        <v>1.47869492596106</v>
+        <v>1.345199956565148</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -1159,38 +1159,38 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>U03</t>
+          <t>U05</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>BAT-A-06</t>
+          <t>BAT-B-01</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1654.859398321596</v>
+        <v>3718.536241088956</v>
       </c>
       <c r="F16" t="n">
-        <v>2014.859398321596</v>
+        <v>4078.536241088956</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>S009</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>3343.473273034984</v>
+        <v>5234.711103060539</v>
       </c>
       <c r="I16" t="n">
-        <v>2.254800043434852</v>
+        <v>1.771485518965449</v>
       </c>
       <c r="J16" t="n">
-        <v>1.345199956565148</v>
+        <v>1.428514481034552</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -1207,24 +1207,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>U01</t>
+          <t>U06</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>BAT-A-04</t>
+          <t>BAT-B-03</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2121.702052162075</v>
+        <v>4955.85023490357</v>
       </c>
       <c r="F17" t="n">
-        <v>2674.776276436764</v>
+        <v>5285.85023490357</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1232,19 +1232,19 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>3533.851197556082</v>
+        <v>6021.321887131056</v>
       </c>
       <c r="I17" t="n">
-        <v>1.150804674846841</v>
+        <v>0.9352874452403556</v>
       </c>
       <c r="J17" t="n">
-        <v>2.44919532515316</v>
+        <v>2.264712554759645</v>
       </c>
       <c r="K17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L17" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18">
@@ -1265,14 +1265,14 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>BAT-C-01</t>
+          <t>BAT-C-03</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2989.729917819312</v>
+        <v>1494.170391878965</v>
       </c>
       <c r="F18" t="n">
-        <v>3439.729917819312</v>
+        <v>1944.170391878965</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>5031.541936458019</v>
+        <v>3535.982410517673</v>
       </c>
       <c r="I18" t="n">
         <v>5.721185016831143</v>
@@ -1313,34 +1313,34 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>BAT-C-02</t>
+          <t>BAT-C-04</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>3759.882476471139</v>
+        <v>1560.170391878965</v>
       </c>
       <c r="F19" t="n">
-        <v>4239.882476471139</v>
+        <v>1980.170391878965</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>6177.316588337516</v>
+        <v>2989.729917819312</v>
       </c>
       <c r="I19" t="n">
-        <v>6.141502088085912</v>
+        <v>2.327805455709593</v>
       </c>
       <c r="J19" t="n">
-        <v>0.2584979119140884</v>
+        <v>4.072194544290408</v>
       </c>
       <c r="K19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L19" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>U08</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1361,34 +1361,34 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>BAT-C-03</t>
+          <t>BAT-C-01</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>5031.541936458019</v>
+        <v>2989.729917819312</v>
       </c>
       <c r="F20" t="n">
-        <v>5421.541936458019</v>
+        <v>3469.729917819312</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>6788.860523942633</v>
+        <v>5407.164029685689</v>
       </c>
       <c r="I20" t="n">
-        <v>3.14468963084745</v>
+        <v>6.141502088085912</v>
       </c>
       <c r="J20" t="n">
-        <v>3.25531036915255</v>
+        <v>0.2584979119140884</v>
       </c>
       <c r="K20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L20" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U08</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1409,34 +1409,34 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>BAT-C-04</t>
+          <t>BAT-C-02</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>6177.316588337516</v>
+        <v>3535.982410517673</v>
       </c>
       <c r="F21" t="n">
-        <v>6597.316588337516</v>
+        <v>3925.982410517673</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>8346.377654930679</v>
+        <v>5293.300998002287</v>
       </c>
       <c r="I21" t="n">
-        <v>5.518469288797766</v>
+        <v>3.14468963084745</v>
       </c>
       <c r="J21" t="n">
-        <v>0.8815307112022346</v>
+        <v>3.25531036915255</v>
       </c>
       <c r="K21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22">
@@ -1457,28 +1457,28 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>BAT-C-01</t>
+          <t>BAT-C-04</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>6788.860523942633</v>
+        <v>5293.300998002287</v>
       </c>
       <c r="F22" t="n">
-        <v>7414.362878516455</v>
+        <v>5713.300998002287</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>8739.558036711996</v>
+        <v>7462.362064595451</v>
       </c>
       <c r="I22" t="n">
-        <v>3.787046244038005</v>
+        <v>5.518469288797766</v>
       </c>
       <c r="J22" t="n">
-        <v>2.612953755961996</v>
+        <v>0.8815307112022346</v>
       </c>
       <c r="K22" t="n">
         <v>4</v>
@@ -1495,44 +1495,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>U06</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>BAT-B-02</t>
+          <t>BAT-C-03</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>3822.018709443888</v>
+        <v>5407.164029685689</v>
       </c>
       <c r="F23" t="n">
-        <v>4152.018709443888</v>
+        <v>5918.803352576108</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>S010</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>5257.395611890227</v>
+        <v>7596.515437168282</v>
       </c>
       <c r="I23" t="n">
-        <v>1.515576193693967</v>
+        <v>5.401510008542074</v>
       </c>
       <c r="J23" t="n">
-        <v>1.684423806306033</v>
+        <v>0.9984899914579266</v>
       </c>
       <c r="K23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L23" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24">
@@ -1543,44 +1543,44 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>U06</t>
+          <t>U08</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>BAT-B-03</t>
+          <t>BAT-C-02</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>5257.395611890227</v>
+        <v>7462.362064595451</v>
       </c>
       <c r="F24" t="n">
-        <v>5587.395611890227</v>
+        <v>7882.362064595451</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>S012</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>7058.749035861612</v>
+        <v>9207.557222790992</v>
       </c>
       <c r="I24" t="n">
-        <v>2.288992826923215</v>
+        <v>3.787046244038005</v>
       </c>
       <c r="J24" t="n">
-        <v>0.911007173076785</v>
+        <v>2.612953755961996</v>
       </c>
       <c r="K24" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L24" t="n">
-        <v>8</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25">
@@ -1605,24 +1605,24 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>5618.325516700729</v>
+        <v>5234.711103060539</v>
       </c>
       <c r="F25" t="n">
-        <v>5948.325516700729</v>
+        <v>5564.711103060539</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>S013</t>
+          <t>S010</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>7006.151204708518</v>
+        <v>6670.088005506878</v>
       </c>
       <c r="I25" t="n">
-        <v>1.514657454833644</v>
+        <v>1.515576193693967</v>
       </c>
       <c r="J25" t="n">
-        <v>1.685342545166356</v>
+        <v>1.684423806306033</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
@@ -1639,44 +1639,44 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>U02</t>
+          <t>U06</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>BAT-A-03</t>
+          <t>BAT-B-02</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2430.151333022899</v>
+        <v>6021.321887131056</v>
       </c>
       <c r="F26" t="n">
-        <v>2760.151333022899</v>
+        <v>6622.164768881158</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S012</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>3621.052478287457</v>
+        <v>8093.518192852543</v>
       </c>
       <c r="I26" t="n">
-        <v>1.178055595164168</v>
+        <v>2.288992826923215</v>
       </c>
       <c r="J26" t="n">
-        <v>2.421944404835832</v>
+        <v>0.911007173076785</v>
       </c>
       <c r="K26" t="n">
         <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27">
@@ -1701,24 +1701,24 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>7006.151204708518</v>
+        <v>6670.088005506878</v>
       </c>
       <c r="F27" t="n">
-        <v>7336.151204708518</v>
+        <v>7000.088005506878</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>S009</t>
+          <t>S013</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>8444.593452102927</v>
+        <v>8057.913693514667</v>
       </c>
       <c r="I27" t="n">
-        <v>1.742426224062348</v>
+        <v>1.514657454833644</v>
       </c>
       <c r="J27" t="n">
-        <v>1.457573775937653</v>
+        <v>1.685342545166356</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
@@ -1735,43 +1735,187 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>U05</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>BAT-B-03</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>8057.913693514667</v>
+      </c>
+      <c r="F28" t="n">
+        <v>8387.913693514667</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>S014</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>9807.665888133684</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1.784481831712911</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1.415518168287089</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1</v>
+      </c>
+      <c r="L28" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>M028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>U02</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>BAT-A-04</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2652.617556574498</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2982.617556574498</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>3843.518701839057</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1.178055595164168</v>
+      </c>
+      <c r="J29" t="n">
+        <v>2.421944404835832</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1</v>
+      </c>
+      <c r="L29" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>M029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>U06</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>BAT-B-02</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>7058.749035861612</v>
-      </c>
-      <c r="F28" t="n">
-        <v>7388.749035861612</v>
-      </c>
-      <c r="G28" t="inlineStr">
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>BAT-B-04</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>8093.518192852543</v>
+      </c>
+      <c r="F30" t="n">
+        <v>8423.518192852544</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>S009</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>9531.960440246952</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1.742426224062348</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1.457573775937653</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1</v>
+      </c>
+      <c r="L30" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>M030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>U06</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>BAT-B-01</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>9531.960440246952</v>
+      </c>
+      <c r="F31" t="n">
+        <v>9861.960440246952</v>
+      </c>
+      <c r="G31" t="inlineStr">
         <is>
           <t>S011</t>
         </is>
       </c>
-      <c r="H28" t="n">
-        <v>8124.220688089099</v>
-      </c>
-      <c r="I28" t="n">
+      <c r="H31" t="n">
+        <v>10597.43209247444</v>
+      </c>
+      <c r="I31" t="n">
         <v>0.8932052893717091</v>
       </c>
-      <c r="J28" t="n">
+      <c r="J31" t="n">
         <v>2.306794710628292</v>
       </c>
-      <c r="K28" t="n">
-        <v>1</v>
-      </c>
-      <c r="L28" t="n">
+      <c r="K31" t="n">
+        <v>1</v>
+      </c>
+      <c r="L31" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1839,7 +1983,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>S007-WAT-01</t>
+          <t>S012-WAT-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1849,11 +1993,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S012</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1163.91968119359</v>
+        <v>1656.230483934338</v>
       </c>
       <c r="E2" t="n">
         <v>3600</v>
@@ -1868,13 +2012,13 @@
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>0.323311022553775</v>
+        <v>0.4600640233150938</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>S007-MED-01</t>
+          <t>S012-MED-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1884,14 +2028,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S012</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1163.91968119359</v>
+        <v>1656.230483934338</v>
       </c>
       <c r="E3" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="F3" t="n">
         <v>3600</v>
@@ -1903,13 +2047,13 @@
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>0.323311022553775</v>
+        <v>0.2300320116575469</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>S006-MED-01</t>
+          <t>S001-MED-02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1919,17 +2063,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1743.722752196917</v>
+        <v>908.5739059656128</v>
       </c>
       <c r="E4" t="n">
         <v>3600</v>
       </c>
       <c r="F4" t="n">
-        <v>3600</v>
+        <v/>
       </c>
       <c r="G4" t="n">
         <v>3600</v>
@@ -1938,13 +2082,13 @@
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>0.4843674311658102</v>
+        <v>0.2523816405460035</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>S012-WAT-01</t>
+          <t>S014-WAT-01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1954,11 +2098,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>S012</t>
+          <t>S014</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1656.230483934338</v>
+        <v>1302.758933892745</v>
       </c>
       <c r="E5" t="n">
         <v>3600</v>
@@ -1973,13 +2117,13 @@
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>0.4600640233150938</v>
+        <v>0.3618774816368735</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S012-MED-01</t>
+          <t>S014-MED-01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1989,11 +2133,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>S012</t>
+          <t>S014</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1656.230483934338</v>
+        <v>1302.758933892745</v>
       </c>
       <c r="E6" t="n">
         <v>7200</v>
@@ -2008,13 +2152,13 @@
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2300320116575469</v>
+        <v>0.1809387408184367</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>S001-MED-02</t>
+          <t>S011-MED-01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2024,32 +2168,32 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S011</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>908.5739059656128</v>
+        <v>2325.266762681505</v>
       </c>
       <c r="E7" t="n">
-        <v>3600</v>
+        <v>10800</v>
       </c>
       <c r="F7" t="n">
-        <v/>
+        <v>10800</v>
       </c>
       <c r="G7" t="n">
-        <v>3600</v>
+        <v>10800</v>
       </c>
       <c r="H7" t="b">
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>0.2523816405460035</v>
+        <v>0.2153024780260653</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>S001-WAT-08</t>
+          <t>S001-WAT-02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2084,7 +2228,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>S001-FOD-02</t>
+          <t>S001-WAT-06</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2101,7 +2245,7 @@
         <v>1248.270195939482</v>
       </c>
       <c r="E9" t="n">
-        <v>7200</v>
+        <v>3600</v>
       </c>
       <c r="F9" t="n">
         <v/>
@@ -2113,13 +2257,13 @@
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1733708605471503</v>
+        <v>0.3467417210943007</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S001-FOD-03</t>
+          <t>S001-WAT-01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2136,25 +2280,25 @@
         <v>1248.270195939482</v>
       </c>
       <c r="E10" t="n">
-        <v>7200</v>
+        <v>3600</v>
       </c>
       <c r="F10" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="G10" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="H10" t="b">
         <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1733708605471503</v>
+        <v>0.3467417210943007</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S001-HYG-01</t>
+          <t>S001-FOD-02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2171,7 +2315,7 @@
         <v>1248.270195939482</v>
       </c>
       <c r="E11" t="n">
-        <v>10800</v>
+        <v>7200</v>
       </c>
       <c r="F11" t="n">
         <v/>
@@ -2183,13 +2327,13 @@
         <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>0.1155805736981002</v>
+        <v>0.1733708605471503</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S001-WAT-07</t>
+          <t>S001-FOD-01</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2206,7 +2350,7 @@
         <v>1248.270195939482</v>
       </c>
       <c r="E12" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="F12" t="n">
         <v/>
@@ -2218,13 +2362,13 @@
         <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>0.3467417210943007</v>
+        <v>0.1733708605471503</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>S001-MED-01</t>
+          <t>S001-FOD-03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2241,25 +2385,25 @@
         <v>1248.270195939482</v>
       </c>
       <c r="E13" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="F13" t="n">
-        <v>3600</v>
+        <v/>
       </c>
       <c r="G13" t="n">
-        <v>3600</v>
+        <v/>
       </c>
       <c r="H13" t="b">
         <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>0.3467417210943007</v>
+        <v>0.1733708605471503</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>S001-WAT-02</t>
+          <t>S001-HYG-01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2276,7 +2420,7 @@
         <v>1248.270195939482</v>
       </c>
       <c r="E14" t="n">
-        <v>3600</v>
+        <v>10800</v>
       </c>
       <c r="F14" t="n">
         <v/>
@@ -2288,13 +2432,13 @@
         <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>0.3467417210943007</v>
+        <v>0.1155805736981002</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>S014-WAT-01</t>
+          <t>S002-WAT-01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2304,11 +2448,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>S014</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1242.432763976175</v>
+        <v>1220.286966960956</v>
       </c>
       <c r="E15" t="n">
         <v>3600</v>
@@ -2323,13 +2467,13 @@
         <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>0.3451202122156041</v>
+        <v>0.3389686019335988</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>S014-MED-01</t>
+          <t>S002-MED-01</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2339,14 +2483,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>S014</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1242.432763976175</v>
+        <v>1220.286966960956</v>
       </c>
       <c r="E16" t="n">
-        <v>7200</v>
+        <v>3600</v>
       </c>
       <c r="F16" t="n">
         <v>3600</v>
@@ -2358,13 +2502,13 @@
         <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>0.172560106107802</v>
+        <v>0.3389686019335988</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>S014-FOD-01</t>
+          <t>S002-FOD-02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2374,11 +2518,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>S014</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1242.432763976175</v>
+        <v>1220.286966960956</v>
       </c>
       <c r="E17" t="n">
         <v>7200</v>
@@ -2393,13 +2537,13 @@
         <v>1</v>
       </c>
       <c r="I17" t="n">
-        <v>0.172560106107802</v>
+        <v>0.1694843009667994</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>S002-WAT-01</t>
+          <t>S001-WAT-08</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2409,32 +2553,32 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1220.286966960956</v>
+        <v>1182.270195939482</v>
       </c>
       <c r="E18" t="n">
         <v>3600</v>
       </c>
       <c r="F18" t="n">
-        <v>3600</v>
+        <v/>
       </c>
       <c r="G18" t="n">
-        <v>3600</v>
+        <v/>
       </c>
       <c r="H18" t="b">
         <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>0.3389686019335988</v>
+        <v>0.3284083877609673</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>S002-MED-01</t>
+          <t>S001-MED-01</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2444,11 +2588,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1220.286966960956</v>
+        <v>1182.270195939482</v>
       </c>
       <c r="E19" t="n">
         <v>3600</v>
@@ -2463,13 +2607,13 @@
         <v>1</v>
       </c>
       <c r="I19" t="n">
-        <v>0.3389686019335988</v>
+        <v>0.3284083877609673</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>S002-FOD-01</t>
+          <t>S001-WAT-05</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2479,14 +2623,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1220.286966960956</v>
+        <v>1182.270195939482</v>
       </c>
       <c r="E20" t="n">
-        <v>7200</v>
+        <v>3600</v>
       </c>
       <c r="F20" t="n">
         <v/>
@@ -2498,7 +2642,7 @@
         <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1694843009667994</v>
+        <v>0.3284083877609673</v>
       </c>
     </row>
     <row r="21">
@@ -2509,7 +2653,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>M006</t>
+          <t>M005</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2539,12 +2683,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>S001-WAT-05</t>
+          <t>S001-WAT-04</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>M006</t>
+          <t>M005</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2574,12 +2718,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>S001-FOD-01</t>
+          <t>S001-WAT-07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>M006</t>
+          <t>M005</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2591,7 +2735,7 @@
         <v>1182.270195939482</v>
       </c>
       <c r="E23" t="n">
-        <v>7200</v>
+        <v>3600</v>
       </c>
       <c r="F23" t="n">
         <v/>
@@ -2603,13 +2747,13 @@
         <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>0.1642041938804836</v>
+        <v>0.3284083877609673</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>S001-WAT-01</t>
+          <t>S007-WAT-01</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2619,11 +2763,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1182.270195939482</v>
+        <v>1133.91968119359</v>
       </c>
       <c r="E24" t="n">
         <v>3600</v>
@@ -2638,13 +2782,13 @@
         <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>0.3284083877609673</v>
+        <v>0.3149776892204416</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>S001-WAT-04</t>
+          <t>S007-MED-01</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2654,67 +2798,67 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1182.270195939482</v>
+        <v>1133.91968119359</v>
       </c>
       <c r="E25" t="n">
         <v>3600</v>
       </c>
       <c r="F25" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="G25" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="H25" t="b">
         <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>0.3284083877609673</v>
+        <v>0.3149776892204416</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>S001-WAT-06</t>
+          <t>S010-WAT-01</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>M006</t>
+          <t>M007</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S010</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1182.270195939482</v>
+        <v>1104.966365827464</v>
       </c>
       <c r="E26" t="n">
         <v>3600</v>
       </c>
       <c r="F26" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="G26" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="H26" t="b">
         <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>0.3284083877609673</v>
+        <v>0.3069351016187401</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>S006-WAT-02</t>
+          <t>S010-MED-01</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2724,107 +2868,107 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S010</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2637.595154849138</v>
+        <v>1104.966365827464</v>
       </c>
       <c r="E27" t="n">
         <v>3600</v>
       </c>
       <c r="F27" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="G27" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="H27" t="b">
         <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>0.7326653207914273</v>
+        <v>0.3069351016187401</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>S006-WAT-03</t>
+          <t>S013-MED-01</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>M007</t>
+          <t>M008</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S013</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2637.595154849138</v>
+        <v>2737.126026344856</v>
       </c>
       <c r="E28" t="n">
         <v>3600</v>
       </c>
       <c r="F28" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="G28" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="H28" t="b">
         <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>0.7326653207914273</v>
+        <v>0.7603127850957931</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>S006-FOD-01</t>
+          <t>S013-WAT-01</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>M007</t>
+          <t>M008</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S013</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2637.595154849138</v>
+        <v>2737.126026344856</v>
       </c>
       <c r="E29" t="n">
-        <v>7200</v>
+        <v>3600</v>
       </c>
       <c r="F29" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="G29" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="H29" t="b">
         <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>0.3663326603957136</v>
+        <v>0.7603127850957931</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>S006-HYG-01</t>
+          <t>S006-WAT-01</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>M007</t>
+          <t>M009</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2833,33 +2977,33 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2637.595154849138</v>
+        <v>882.4017897442618</v>
       </c>
       <c r="E30" t="n">
-        <v>10800</v>
+        <v>3600</v>
       </c>
       <c r="F30" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="G30" t="n">
-        <v/>
+        <v>3600</v>
       </c>
       <c r="H30" t="b">
         <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>0.2442217735971424</v>
+        <v>0.2451116082622949</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>S006-WAT-01</t>
+          <t>S006-MED-01</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>M007</t>
+          <t>M009</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2868,7 +3012,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2637.595154849138</v>
+        <v>882.4017897442618</v>
       </c>
       <c r="E31" t="n">
         <v>3600</v>
@@ -2883,158 +3027,158 @@
         <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>0.7326653207914273</v>
+        <v>0.2451116082622949</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>S010-WAT-01</t>
+          <t>S003-WAT-01</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>M008</t>
+          <t>M010</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>S010</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1104.966365827464</v>
+        <v>3114.250545432328</v>
       </c>
       <c r="E32" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="F32" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="G32" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="H32" t="b">
         <v>1</v>
       </c>
       <c r="I32" t="n">
-        <v>0.3069351016187401</v>
+        <v>0.4325347979767122</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>S010-MED-01</t>
+          <t>S003-MED-01</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>M008</t>
+          <t>M010</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>S010</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1104.966365827464</v>
+        <v>3114.250545432328</v>
       </c>
       <c r="E33" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="F33" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="G33" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="H33" t="b">
         <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>0.3069351016187401</v>
+        <v>0.4325347979767122</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>S013-WAT-01</t>
+          <t>S004-WAT-01</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>M009</t>
+          <t>M011</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>S013</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1082.266628023259</v>
+        <v>2449.747585075144</v>
       </c>
       <c r="E34" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="F34" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="G34" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="H34" t="b">
         <v>1</v>
       </c>
       <c r="I34" t="n">
-        <v>0.3006296188953499</v>
+        <v>0.3402427201493256</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>S013-MED-01</t>
+          <t>S004-MED-01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>M009</t>
+          <t>M011</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>S013</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1082.266628023259</v>
+        <v>2449.747585075144</v>
       </c>
       <c r="E35" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="F35" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="G35" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="H35" t="b">
         <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>0.3006296188953499</v>
+        <v>0.3402427201493256</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>S008-WAT-01</t>
+          <t>S008-MED-01</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>M010</t>
+          <t>M012</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3043,7 +3187,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>3057.866434175052</v>
+        <v>3047.8417541721</v>
       </c>
       <c r="E36" t="n">
         <v>7200</v>
@@ -3058,18 +3202,18 @@
         <v>1</v>
       </c>
       <c r="I36" t="n">
-        <v>0.4247036714132016</v>
+        <v>0.423311354746125</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>S008-MED-01</t>
+          <t>S008-WAT-01</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>M010</t>
+          <t>M012</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3078,7 +3222,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>3057.866434175052</v>
+        <v>3047.8417541721</v>
       </c>
       <c r="E37" t="n">
         <v>7200</v>
@@ -3093,97 +3237,97 @@
         <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>0.4247036714132016</v>
+        <v>0.423311354746125</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>S008-WAT-02</t>
+          <t>S015-MED-01</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>M010</t>
+          <t>M013</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>S015</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>3057.866434175052</v>
+        <v>4345.827579449335</v>
       </c>
       <c r="E38" t="n">
         <v>7200</v>
       </c>
       <c r="F38" t="n">
-        <v/>
+        <v>7200</v>
       </c>
       <c r="G38" t="n">
-        <v/>
+        <v>7200</v>
       </c>
       <c r="H38" t="b">
         <v>1</v>
       </c>
       <c r="I38" t="n">
-        <v>0.4247036714132016</v>
+        <v>0.6035871638124076</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>S008-FOD-01</t>
+          <t>S015-WAT-01</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>M010</t>
+          <t>M013</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>S015</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>3057.866434175052</v>
+        <v>4345.827579449335</v>
       </c>
       <c r="E39" t="n">
         <v>10800</v>
       </c>
       <c r="F39" t="n">
-        <v/>
+        <v>10800</v>
       </c>
       <c r="G39" t="n">
-        <v/>
+        <v>10800</v>
       </c>
       <c r="H39" t="b">
         <v>1</v>
       </c>
       <c r="I39" t="n">
-        <v>0.2831357809421344</v>
+        <v>0.4023914425416051</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>S008-HYG-01</t>
+          <t>S015-FOD-01</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>M010</t>
+          <t>M013</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>S015</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>3057.866434175052</v>
+        <v>4345.827579449335</v>
       </c>
       <c r="E40" t="n">
         <v>14400</v>
@@ -3198,240 +3342,240 @@
         <v>1</v>
       </c>
       <c r="I40" t="n">
-        <v>0.2123518357066008</v>
+        <v>0.3017935819062038</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>S003-WAT-01</t>
+          <t>S009-WAT-01</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>M011</t>
+          <t>M014</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S009</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>3097.329655016233</v>
+        <v>3556.048270379593</v>
       </c>
       <c r="E41" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="F41" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="G41" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="H41" t="b">
         <v>1</v>
       </c>
       <c r="I41" t="n">
-        <v>0.4301846743078101</v>
+        <v>0.3292637287388512</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>S003-MED-01</t>
+          <t>S009-MED-01</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>M011</t>
+          <t>M014</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S009</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3097.329655016233</v>
+        <v>3556.048270379593</v>
       </c>
       <c r="E42" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="F42" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="G42" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="H42" t="b">
         <v>1</v>
       </c>
       <c r="I42" t="n">
-        <v>0.4301846743078101</v>
+        <v>0.3292637287388512</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>S004-WAT-01</t>
+          <t>S005-WAT-01</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>M012</t>
+          <t>M015</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3112.222866872304</v>
+        <v>4759.380338741414</v>
       </c>
       <c r="E43" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="F43" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="G43" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="H43" t="b">
         <v>1</v>
       </c>
       <c r="I43" t="n">
-        <v>0.4322531759544866</v>
+        <v>0.440683364698279</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>S004-MED-01</t>
+          <t>S005-MED-01</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>M012</t>
+          <t>M015</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>3112.222866872304</v>
+        <v>4759.380338741414</v>
       </c>
       <c r="E44" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="F44" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="G44" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="H44" t="b">
         <v>1</v>
       </c>
       <c r="I44" t="n">
-        <v>0.4322531759544866</v>
+        <v>0.440683364698279</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>S015-MED-01</t>
+          <t>S011-WAT-01</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>M013</t>
+          <t>M016</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>S015</t>
+          <t>S011</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>5008.302861246493</v>
+        <v>5740.77272768398</v>
       </c>
       <c r="E45" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="F45" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="G45" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="H45" t="b">
         <v>1</v>
       </c>
       <c r="I45" t="n">
-        <v>0.6955976196175685</v>
+        <v>0.5315530303411092</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>S015-WAT-01</t>
+          <t>S002-WAT-03</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>M013</t>
+          <t>M017</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>S015</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>5008.302861246493</v>
+        <v>2915.486401198319</v>
       </c>
       <c r="E46" t="n">
-        <v>10800</v>
+        <v>3600</v>
       </c>
       <c r="F46" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="G46" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="H46" t="b">
         <v>1</v>
       </c>
       <c r="I46" t="n">
-        <v>0.4637317464117123</v>
+        <v>0.8098573336661997</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>S015-FOD-01</t>
+          <t>S002-FOD-01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>M013</t>
+          <t>M017</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>S015</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>5008.302861246493</v>
+        <v>2915.486401198319</v>
       </c>
       <c r="E47" t="n">
-        <v>14400</v>
+        <v>7200</v>
       </c>
       <c r="F47" t="n">
         <v/>
@@ -3443,240 +3587,240 @@
         <v>1</v>
       </c>
       <c r="I47" t="n">
-        <v>0.3477988098087842</v>
+        <v>0.4049286668330998</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>S005-WAT-01</t>
+          <t>S002-HYG-01</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>M014</t>
+          <t>M017</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2738.321381855582</v>
+        <v>2915.486401198319</v>
       </c>
       <c r="E48" t="n">
         <v>10800</v>
       </c>
       <c r="F48" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="G48" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="H48" t="b">
         <v>1</v>
       </c>
       <c r="I48" t="n">
-        <v>0.2535482760977391</v>
+        <v>0.2699524445553999</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>S005-MED-01</t>
+          <t>S002-WAT-02</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>M014</t>
+          <t>M017</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>2738.321381855582</v>
+        <v>2915.486401198319</v>
       </c>
       <c r="E49" t="n">
-        <v>10800</v>
+        <v>3600</v>
       </c>
       <c r="F49" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="G49" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="H49" t="b">
         <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>0.2535482760977391</v>
+        <v>0.8098573336661997</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>S009-WAT-01</t>
+          <t>S002-WAT-04</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>M015</t>
+          <t>M017</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>S009</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>2780.75633567829</v>
+        <v>2915.486401198319</v>
       </c>
       <c r="E50" t="n">
-        <v>10800</v>
+        <v>3600</v>
       </c>
       <c r="F50" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="G50" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="H50" t="b">
         <v>1</v>
       </c>
       <c r="I50" t="n">
-        <v>0.2574774384887305</v>
+        <v>0.8098573336661997</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>S009-MED-01</t>
+          <t>S006-WAT-02</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>M015</t>
+          <t>M018</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>S009</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2780.75633567829</v>
+        <v>2637.595154849138</v>
       </c>
       <c r="E51" t="n">
-        <v>10800</v>
+        <v>3600</v>
       </c>
       <c r="F51" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="G51" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="H51" t="b">
         <v>1</v>
       </c>
       <c r="I51" t="n">
-        <v>0.2574774384887305</v>
+        <v>0.7326653207914273</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>S011-WAT-01</t>
+          <t>S006-WAT-03</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>M016</t>
+          <t>M018</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>S011</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>3206.500403663089</v>
+        <v>2637.595154849138</v>
       </c>
       <c r="E52" t="n">
-        <v>10800</v>
+        <v>3600</v>
       </c>
       <c r="F52" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="G52" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="H52" t="b">
         <v>1</v>
       </c>
       <c r="I52" t="n">
-        <v>0.2968981855243601</v>
+        <v>0.7326653207914273</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S011-MED-01</t>
+          <t>S006-FOD-01</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>M016</t>
+          <t>M018</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>S011</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>3206.500403663089</v>
+        <v>2637.595154849138</v>
       </c>
       <c r="E53" t="n">
-        <v>10800</v>
+        <v>7200</v>
       </c>
       <c r="F53" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="G53" t="n">
-        <v>10800</v>
+        <v/>
       </c>
       <c r="H53" t="b">
         <v>1</v>
       </c>
       <c r="I53" t="n">
-        <v>0.2968981855243601</v>
+        <v>0.3663326603957136</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>S002-WAT-02</t>
+          <t>S006-HYG-01</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>M017</t>
+          <t>M018</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>4411.045927138666</v>
+        <v>2637.595154849138</v>
       </c>
       <c r="E54" t="n">
-        <v>3600</v>
+        <v>10800</v>
       </c>
       <c r="F54" t="n">
         <v/>
@@ -3688,30 +3832,30 @@
         <v>1</v>
       </c>
       <c r="I54" t="n">
-        <v>1.225290535316296</v>
+        <v>0.2442217735971424</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>S002-WAT-03</t>
+          <t>S003-WAT-02</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>M017</t>
+          <t>M019</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>4411.045927138666</v>
+        <v>4625.906973752501</v>
       </c>
       <c r="E55" t="n">
-        <v>3600</v>
+        <v>7200</v>
       </c>
       <c r="F55" t="n">
         <v/>
@@ -3723,27 +3867,27 @@
         <v>1</v>
       </c>
       <c r="I55" t="n">
-        <v>1.225290535316296</v>
+        <v>0.6424870796878474</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>S002-FOD-02</t>
+          <t>S003-WAT-03</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>M017</t>
+          <t>M019</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>4411.045927138666</v>
+        <v>4625.906973752501</v>
       </c>
       <c r="E56" t="n">
         <v>7200</v>
@@ -3758,30 +3902,30 @@
         <v>1</v>
       </c>
       <c r="I56" t="n">
-        <v>0.6126452676581481</v>
+        <v>0.6424870796878474</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>S002-HYG-01</t>
+          <t>S003-WAT-04</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>M017</t>
+          <t>M019</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>4411.045927138666</v>
+        <v>4625.906973752501</v>
       </c>
       <c r="E57" t="n">
-        <v>10800</v>
+        <v>7200</v>
       </c>
       <c r="F57" t="n">
         <v/>
@@ -3793,30 +3937,30 @@
         <v>1</v>
       </c>
       <c r="I57" t="n">
-        <v>0.4084301784387654</v>
+        <v>0.6424870796878474</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>S002-WAT-04</t>
+          <t>S003-FOD-01</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>M017</t>
+          <t>M019</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>4411.045927138666</v>
+        <v>4625.906973752501</v>
       </c>
       <c r="E58" t="n">
-        <v>3600</v>
+        <v>10800</v>
       </c>
       <c r="F58" t="n">
         <v/>
@@ -3828,18 +3972,18 @@
         <v>1</v>
       </c>
       <c r="I58" t="n">
-        <v>1.225290535316296</v>
+        <v>0.4283247197918982</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>S003-WAT-02</t>
+          <t>S003-FOD-02</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>M018</t>
+          <t>M019</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3848,10 +3992,10 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>5396.059532404328</v>
+        <v>4625.906973752501</v>
       </c>
       <c r="E59" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="F59" t="n">
         <v/>
@@ -3863,18 +4007,18 @@
         <v>1</v>
       </c>
       <c r="I59" t="n">
-        <v>0.7494527128339344</v>
+        <v>0.4283247197918982</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>S003-WAT-03</t>
+          <t>S003-HYG-01</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>M018</t>
+          <t>M019</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3883,10 +4027,10 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>5396.059532404328</v>
+        <v>4625.906973752501</v>
       </c>
       <c r="E60" t="n">
-        <v>7200</v>
+        <v>14400</v>
       </c>
       <c r="F60" t="n">
         <v/>
@@ -3898,30 +4042,30 @@
         <v>1</v>
       </c>
       <c r="I60" t="n">
-        <v>0.7494527128339344</v>
+        <v>0.3212435398439237</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>S003-WAT-04</t>
+          <t>S007-WAT-02</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>M018</t>
+          <t>M020</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>5396.059532404328</v>
+        <v>4742.60170425998</v>
       </c>
       <c r="E61" t="n">
-        <v>7200</v>
+        <v>3600</v>
       </c>
       <c r="F61" t="n">
         <v/>
@@ -3933,30 +4077,30 @@
         <v>1</v>
       </c>
       <c r="I61" t="n">
-        <v>0.7494527128339344</v>
+        <v>1.317389362294439</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>S003-FOD-01</t>
+          <t>S007-FOD-01</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>M018</t>
+          <t>M020</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>5396.059532404328</v>
+        <v>4742.60170425998</v>
       </c>
       <c r="E62" t="n">
-        <v>10800</v>
+        <v>7200</v>
       </c>
       <c r="F62" t="n">
         <v/>
@@ -3968,27 +4112,27 @@
         <v>1</v>
       </c>
       <c r="I62" t="n">
-        <v>0.4996351418892896</v>
+        <v>0.6586946811472194</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>S003-FOD-02</t>
+          <t>S007-HYG-01</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>M018</t>
+          <t>M020</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>5396.059532404328</v>
+        <v>4742.60170425998</v>
       </c>
       <c r="E63" t="n">
         <v>10800</v>
@@ -4003,30 +4147,30 @@
         <v>1</v>
       </c>
       <c r="I63" t="n">
-        <v>0.4996351418892896</v>
+        <v>0.4391297874314796</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S003-HYG-01</t>
+          <t>S004-WAT-03</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>M018</t>
+          <t>M021</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5396.059532404328</v>
+        <v>6744.801531298868</v>
       </c>
       <c r="E64" t="n">
-        <v>14400</v>
+        <v>7200</v>
       </c>
       <c r="F64" t="n">
         <v/>
@@ -4038,30 +4182,30 @@
         <v>1</v>
       </c>
       <c r="I64" t="n">
-        <v>0.3747263564169672</v>
+        <v>0.936777990458176</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>S007-WAT-02</t>
+          <t>S004-FOD-01</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>M019</t>
+          <t>M021</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>6238.161230200327</v>
+        <v>6744.801531298868</v>
       </c>
       <c r="E65" t="n">
-        <v>3600</v>
+        <v>10800</v>
       </c>
       <c r="F65" t="n">
         <v/>
@@ -4073,30 +4217,30 @@
         <v>1</v>
       </c>
       <c r="I65" t="n">
-        <v>1.732822563944535</v>
+        <v>0.6245186603054508</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>S007-FOD-01</t>
+          <t>S004-HYG-01</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>M019</t>
+          <t>M021</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>6238.161230200327</v>
+        <v>6744.801531298868</v>
       </c>
       <c r="E66" t="n">
-        <v>7200</v>
+        <v>14400</v>
       </c>
       <c r="F66" t="n">
         <v/>
@@ -4108,30 +4252,30 @@
         <v>1</v>
       </c>
       <c r="I66" t="n">
-        <v>0.8664112819722676</v>
+        <v>0.468388995229088</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>S007-HYG-01</t>
+          <t>S004-WAT-02</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>M019</t>
+          <t>M021</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>6238.161230200327</v>
+        <v>6744.801531298868</v>
       </c>
       <c r="E67" t="n">
-        <v>10800</v>
+        <v>7200</v>
       </c>
       <c r="F67" t="n">
         <v/>
@@ -4143,27 +4287,27 @@
         <v>1</v>
       </c>
       <c r="I67" t="n">
-        <v>0.5776075213148451</v>
+        <v>0.936777990458176</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>S004-WAT-02</t>
+          <t>S008-WAT-02</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>M020</t>
+          <t>M022</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>7628.817121634098</v>
+        <v>6894.499394872195</v>
       </c>
       <c r="E68" t="n">
         <v>7200</v>
@@ -4178,30 +4322,30 @@
         <v>1</v>
       </c>
       <c r="I68" t="n">
-        <v>1.059557933560291</v>
+        <v>0.957569360398916</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>S004-WAT-03</t>
+          <t>S008-FOD-01</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>M020</t>
+          <t>M022</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>7628.817121634098</v>
+        <v>6894.499394872195</v>
       </c>
       <c r="E69" t="n">
-        <v>7200</v>
+        <v>10800</v>
       </c>
       <c r="F69" t="n">
         <v/>
@@ -4213,30 +4357,30 @@
         <v>1</v>
       </c>
       <c r="I69" t="n">
-        <v>1.059557933560291</v>
+        <v>0.6383795735992773</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>S004-FOD-01</t>
+          <t>S008-HYG-01</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>M020</t>
+          <t>M022</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>7628.817121634098</v>
+        <v>6894.499394872195</v>
       </c>
       <c r="E70" t="n">
-        <v>10800</v>
+        <v>14400</v>
       </c>
       <c r="F70" t="n">
         <v/>
@@ -4248,30 +4392,30 @@
         <v>1</v>
       </c>
       <c r="I70" t="n">
-        <v>0.706371955706861</v>
+        <v>0.4787846801994579</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>S004-HYG-01</t>
+          <t>S005-WAT-02</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>M020</t>
+          <t>M023</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>7628.817121634098</v>
+        <v>8703.594643693221</v>
       </c>
       <c r="E71" t="n">
-        <v>14400</v>
+        <v>10800</v>
       </c>
       <c r="F71" t="n">
         <v/>
@@ -4283,18 +4427,18 @@
         <v>1</v>
       </c>
       <c r="I71" t="n">
-        <v>0.5297789667801457</v>
+        <v>0.8058883929345575</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>S005-WAT-02</t>
+          <t>S005-WAT-03</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>M021</t>
+          <t>M023</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -4303,7 +4447,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>8235.595457614225</v>
+        <v>8703.594643693221</v>
       </c>
       <c r="E72" t="n">
         <v>10800</v>
@@ -4318,18 +4462,18 @@
         <v>1</v>
       </c>
       <c r="I72" t="n">
-        <v>0.7625551349642801</v>
+        <v>0.8058883929345575</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>S005-WAT-03</t>
+          <t>S005-FOD-01</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>M021</t>
+          <t>M023</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -4338,10 +4482,10 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>8235.595457614225</v>
+        <v>8703.594643693221</v>
       </c>
       <c r="E73" t="n">
-        <v>10800</v>
+        <v>14400</v>
       </c>
       <c r="F73" t="n">
         <v/>
@@ -4353,18 +4497,18 @@
         <v>1</v>
       </c>
       <c r="I73" t="n">
-        <v>0.7625551349642801</v>
+        <v>0.6044162947009181</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>S005-FOD-01</t>
+          <t>S005-HYG-01</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>M021</t>
+          <t>M023</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -4373,10 +4517,10 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>8235.595457614225</v>
+        <v>8703.594643693221</v>
       </c>
       <c r="E74" t="n">
-        <v>14400</v>
+        <v>18000</v>
       </c>
       <c r="F74" t="n">
         <v/>
@@ -4388,30 +4532,30 @@
         <v>1</v>
       </c>
       <c r="I74" t="n">
-        <v>0.5719163512232101</v>
+        <v>0.4835330357607345</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>S005-HYG-01</t>
+          <t>S010-FOD-01</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>M021</t>
+          <t>M024</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S010</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>8235.595457614225</v>
+        <v>6199.936220950375</v>
       </c>
       <c r="E75" t="n">
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="F75" t="n">
         <v/>
@@ -4423,27 +4567,27 @@
         <v>1</v>
       </c>
       <c r="I75" t="n">
-        <v>0.457533080978568</v>
+        <v>0.8611022529097744</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>S010-FOD-01</t>
+          <t>S012-FOD-01</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>M022</t>
+          <t>M025</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>S010</t>
+          <t>S012</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>4787.243827333724</v>
+        <v>7442.771480866851</v>
       </c>
       <c r="E76" t="n">
         <v>7200</v>
@@ -4458,27 +4602,27 @@
         <v>1</v>
       </c>
       <c r="I76" t="n">
-        <v>0.6648949760185727</v>
+        <v>1.033718261231507</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>S012-FOD-01</t>
+          <t>S013-FOD-01</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>M023</t>
+          <t>M026</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>S012</t>
+          <t>S013</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>6408.00232387592</v>
+        <v>7611.534182844106</v>
       </c>
       <c r="E77" t="n">
         <v>7200</v>
@@ -4493,27 +4637,27 @@
         <v>1</v>
       </c>
       <c r="I77" t="n">
-        <v>0.8900003227605444</v>
+        <v>1.057157525395015</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>S013-FOD-01</t>
+          <t>S014-FOD-01</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>M024</t>
+          <t>M027</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>S013</t>
+          <t>S014</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>6559.771694037957</v>
+        <v>9180.346457490839</v>
       </c>
       <c r="E78" t="n">
         <v>7200</v>
@@ -4528,7 +4672,7 @@
         <v>1</v>
       </c>
       <c r="I78" t="n">
-        <v>0.9110794019497164</v>
+        <v>1.27504811909595</v>
       </c>
     </row>
     <row r="79">
@@ -4539,7 +4683,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>M025</t>
+          <t>M028</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4548,7 +4692,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>3278.725238988512</v>
+        <v>3501.19146254011</v>
       </c>
       <c r="E79" t="n">
         <v>10800</v>
@@ -4563,7 +4707,7 @@
         <v>1</v>
       </c>
       <c r="I79" t="n">
-        <v>0.303585670276714</v>
+        <v>0.3241843946796399</v>
       </c>
     </row>
     <row r="80">
@@ -4574,7 +4718,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>M026</t>
+          <t>M029</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4583,7 +4727,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>7976.962328405722</v>
+        <v>9064.329316549747</v>
       </c>
       <c r="E80" t="n">
         <v>14400</v>
@@ -4598,7 +4742,7 @@
         <v>1</v>
       </c>
       <c r="I80" t="n">
-        <v>0.5539557172503974</v>
+        <v>0.629467313649288</v>
       </c>
     </row>
     <row r="81">
@@ -4609,7 +4753,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>M027</t>
+          <t>M030</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4618,7 +4762,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>7843.671528642022</v>
+        <v>10316.88293302736</v>
       </c>
       <c r="E81" t="n">
         <v>14400</v>
@@ -4633,7 +4777,7 @@
         <v>1</v>
       </c>
       <c r="I81" t="n">
-        <v>0.5446994117112516</v>
+        <v>0.7164502036824557</v>
       </c>
     </row>
   </sheetData>

</xml_diff>